<commit_message>
Add SOH report for 2026-10-15
</commit_message>
<xml_diff>
--- a/reports/SOH_14_10_2026.xlsx
+++ b/reports/SOH_14_10_2026.xlsx
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-43</v>
+        <v>-42</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>8000</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-57</v>
+        <v>-56</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>8000</v>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>946</v>
+        <v>865</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>3200</v>
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>1112</v>
+        <v>982</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>2900</v>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>929</v>
+        <v>899</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>2800</v>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1520</v>
+        <v>1440</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>2600</v>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>928</v>
+        <v>878</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>3500</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="E54" s="3" t="n">
         <v>5000</v>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>874</v>
+        <v>754</v>
       </c>
       <c r="E55" s="3" t="n">
         <v>4100</v>
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>972</v>
+        <v>592</v>
       </c>
       <c r="E56" s="3" t="n">
         <v>3700</v>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>523</v>
+        <v>223</v>
       </c>
       <c r="E61" s="3" t="n">
         <v>3900</v>
@@ -2281,7 +2281,7 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>956</v>
+        <v>926</v>
       </c>
       <c r="E66" s="3" t="n">
         <v>5000</v>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>5000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E84" s="3" t="n">
         <v>9000</v>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E95" s="3" t="n">
         <v>7612</v>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E96" s="3" t="n">
         <v>8000</v>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>8597</v>
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E99" s="3" t="n">
         <v>8597</v>
@@ -3233,7 +3233,7 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E100" s="3" t="n">
         <v>8597</v>
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E101" s="3" t="n">
         <v>8597</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E103" s="3" t="n">
         <v>4708</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>4708</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" s="3" t="n">
         <v>4708</v>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E106" s="3" t="n">
         <v>12500</v>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E119" s="3" t="n">
         <v>5000</v>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E129" s="3" t="n">
         <v>2500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E137" s="3" t="n">
         <v>3500</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="D235" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E235" s="3" t="n">
         <v>8000</v>
@@ -6953,7 +6953,7 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E236" s="3" t="n">
         <v>6750</v>
@@ -7329,7 +7329,7 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E250" s="3" t="n">
         <v>15851</v>
@@ -8505,7 +8505,7 @@
         </is>
       </c>
       <c r="D292" s="2" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E292" s="3" t="n">
         <v>80577</v>
@@ -9570,7 +9570,7 @@
         </is>
       </c>
       <c r="D330" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E330" s="3" t="n">
         <v>28285</v>
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="D351" s="2" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E351" s="3" t="n">
         <v>9468</v>
@@ -12510,7 +12510,7 @@
         </is>
       </c>
       <c r="D435" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E435" s="3" t="n">
         <v>28285</v>
@@ -12650,7 +12650,7 @@
         </is>
       </c>
       <c r="D440" s="2" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E440" s="3" t="n">
         <v>9967</v>
@@ -12678,7 +12678,7 @@
         </is>
       </c>
       <c r="D441" s="2" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E441" s="3" t="n">
         <v>37711</v>
@@ -12706,7 +12706,7 @@
         </is>
       </c>
       <c r="D442" s="2" t="n">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E442" s="3" t="n">
         <v>37709</v>
@@ -12734,7 +12734,7 @@
         </is>
       </c>
       <c r="D443" s="2" t="n">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E443" s="3" t="n">
         <v>37709</v>
@@ -12762,7 +12762,7 @@
         </is>
       </c>
       <c r="D444" s="2" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E444" s="3" t="n">
         <v>37711</v>
@@ -12902,7 +12902,7 @@
         </is>
       </c>
       <c r="D449" s="2" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E449" s="3" t="n">
         <v>8855.5</v>
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="D452" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E452" s="3" t="n">
         <v>6183</v>
@@ -14414,7 +14414,7 @@
         </is>
       </c>
       <c r="D503" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E503" s="3" t="n">
         <v>3672</v>
@@ -14890,7 +14890,7 @@
         </is>
       </c>
       <c r="D520" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E520" s="3" t="n">
         <v>17379</v>
@@ -16626,7 +16626,7 @@
         </is>
       </c>
       <c r="D582" s="2" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E582" s="3" t="n">
         <v>11436</v>
@@ -17271,7 +17271,7 @@
         </is>
       </c>
       <c r="D605" s="2" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E605" s="3" t="n">
         <v>9932</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>3809</v>
+        <v>3785</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -18895,7 +18895,7 @@
         </is>
       </c>
       <c r="D663" s="2" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E663" s="3" t="n">
         <v>3987</v>
@@ -20043,7 +20043,7 @@
         </is>
       </c>
       <c r="D704" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E704" s="3" t="n">
         <v>40266</v>
@@ -20127,7 +20127,7 @@
         </is>
       </c>
       <c r="D707" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E707" s="3" t="n">
         <v>10923</v>
@@ -20575,7 +20575,7 @@
         </is>
       </c>
       <c r="D723" s="2" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E723" s="3" t="n">
         <v>12992</v>
@@ -22983,7 +22983,7 @@
         </is>
       </c>
       <c r="D809" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E809" s="3" t="n">
         <v>33252</v>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="D825" s="2" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E825" s="3" t="n">
         <v>9932</v>
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="D862" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E862" s="3" t="n">
         <v>33252</v>
@@ -24834,7 +24834,7 @@
         </is>
       </c>
       <c r="D875" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E875" s="3" t="n">
         <v>28285</v>
@@ -24863,7 +24863,7 @@
         </is>
       </c>
       <c r="D876" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E876" s="3" t="n">
         <v>28285</v>
@@ -24892,7 +24892,7 @@
         </is>
       </c>
       <c r="D877" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E877" s="3" t="n">
         <v>32387</v>
@@ -28336,7 +28336,7 @@
         </is>
       </c>
       <c r="D1000" s="2" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E1000" s="3" t="n">
         <v>14215</v>
@@ -29345,7 +29345,7 @@
         </is>
       </c>
       <c r="D1036" s="2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E1036" s="3" t="n">
         <v>9932</v>
@@ -30857,7 +30857,7 @@
         </is>
       </c>
       <c r="D1090" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1090" s="3" t="n">
         <v>9037</v>
@@ -31613,7 +31613,7 @@
         </is>
       </c>
       <c r="D1117" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E1117" s="3" t="n">
         <v>9077</v>
@@ -32201,7 +32201,7 @@
         </is>
       </c>
       <c r="D1138" s="2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E1138" s="3" t="n">
         <v>4651</v>
@@ -35393,7 +35393,7 @@
         </is>
       </c>
       <c r="D1252" s="2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E1252" s="3" t="n">
         <v>28914</v>
@@ -36121,7 +36121,7 @@
         </is>
       </c>
       <c r="D1278" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1278" s="3" t="n">
         <v>34055</v>
@@ -36233,7 +36233,7 @@
         </is>
       </c>
       <c r="D1282" s="2" t="n">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E1282" s="3" t="n">
         <v>8246</v>
@@ -42533,7 +42533,7 @@
         </is>
       </c>
       <c r="D1507" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E1507" s="3" t="n">
         <v>27542</v>
@@ -42701,7 +42701,7 @@
         </is>
       </c>
       <c r="D1513" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1513" s="3" t="n">
         <v>32387</v>
@@ -42758,7 +42758,7 @@
         </is>
       </c>
       <c r="D1515" s="2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E1515" s="3" t="n">
         <v>9932</v>
@@ -43851,7 +43851,7 @@
         </is>
       </c>
       <c r="D1554" s="2" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E1554" s="3" t="n">
         <v>9932</v>

</xml_diff>